<commit_message>
Update Excel files: Future Store List, RBM BDM BRANCH, myG All Store
</commit_message>
<xml_diff>
--- a/Future Store List.xlsx
+++ b/Future Store List.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="9000"/>
+    <workbookView windowWidth="23040" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
   <si>
     <t>Store</t>
   </si>
@@ -206,6 +206,9 @@
   </si>
   <si>
     <t>ATTINGAL FUTURE</t>
+  </si>
+  <si>
+    <t>CHEMMAD FUTURE</t>
   </si>
 </sst>
 </file>
@@ -829,7 +832,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -847,9 +850,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1385,7 +1385,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:A59"/>
+  <dimension ref="A1:A60"/>
   <sheetFormatPr defaultColWidth="9.13888888888889" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="30.712962962963" style="1" customWidth="1"/>
@@ -1677,13 +1677,18 @@
       </c>
     </row>
     <row r="58" spans="1:1">
-      <c r="A58" s="7" t="s">
+      <c r="A58" s="5" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="59" spans="1:1">
-      <c r="A59" s="7" t="s">
+      <c r="A59" s="5" t="s">
         <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1">
+      <c r="A60" s="3" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Excel data files: Future Store List, RBM/BDM/Branch, myG All Store
</commit_message>
<xml_diff>
--- a/Future Store List.xlsx
+++ b/Future Store List.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="8280"/>
+    <workbookView windowWidth="23040" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
   <si>
     <t>Store</t>
   </si>
@@ -213,6 +213,9 @@
   </si>
   <si>
     <t>FALNIR FUTURE</t>
+  </si>
+  <si>
+    <t>THRIPUNITHURA FUTURE</t>
   </si>
 </sst>
 </file>
@@ -836,7 +839,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -858,6 +861,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -872,7 +878,7 @@
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
     <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
     <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
@@ -1392,7 +1398,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:A62"/>
+  <dimension ref="A1:A63"/>
   <sheetFormatPr defaultColWidth="9.13888888888889" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="30.712962962963" style="1" customWidth="1"/>
@@ -1708,6 +1714,11 @@
         <v>61</v>
       </c>
     </row>
+    <row r="63" spans="1:1">
+      <c r="A63" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>